<commit_message>
Update selenium_test_report.xlsx with latest sample run results
</commit_message>
<xml_diff>
--- a/selenium-tests/selenium_test_report.xlsx
+++ b/selenium-tests/selenium_test_report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="39">
   <si>
     <t>SkillSphereAI Web E2E Test Report</t>
   </si>
@@ -23,16 +23,19 @@
     <t>Execution Start</t>
   </si>
   <si>
-    <t>2026-06-17 05:33:03</t>
+    <t>2026-06-17 05:34:38</t>
   </si>
   <si>
     <t>Execution End</t>
   </si>
   <si>
+    <t>2026-06-17 05:35:13</t>
+  </si>
+  <si>
     <t>Total Duration</t>
   </si>
   <si>
-    <t>0.00 seconds</t>
+    <t>35.37 seconds</t>
   </si>
   <si>
     <t>Total Test Steps</t>
@@ -47,7 +50,7 @@
     <t>Pass Rate</t>
   </si>
   <si>
-    <t>100.0%</t>
+    <t>0.0%</t>
   </si>
   <si>
     <t>No.</t>
@@ -74,92 +77,66 @@
     <t>Launch Web Application</t>
   </si>
   <si>
-    <t>PASS</t>
-  </si>
-  <si>
-    <t>Chrome launched. Homepage rendered at http://localhost:3000.</t>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="auth-panel-container"])
+Wait timed out after 12195ms</t>
+  </si>
+  <si>
+    <t>screenshots\fail_launch_web_application_1781674513442.png</t>
+  </si>
+  <si>
+    <t>Authentication / Login</t>
+  </si>
+  <si>
+    <t>SKIP</t>
+  </si>
+  <si>
+    <t>Skipped due to earlier test failure.</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Authentication / Login</t>
-  </si>
-  <si>
-    <t>Credentials entered. OTP bypass 402921 submitted. Dashboard loaded.</t>
-  </si>
-  <si>
     <t>Register New Account (if needed)</t>
   </si>
   <si>
-    <t>User already authenticated. Registration step skipped.</t>
-  </si>
-  <si>
     <t>Onboarding — Demographics</t>
   </si>
   <si>
-    <t>Name field filled and Academics button clicked.</t>
-  </si>
-  <si>
     <t>Onboarding — Academic Details</t>
   </si>
   <si>
-    <t>University, Degree, Major, CGPA filled. Skills page opened.</t>
-  </si>
-  <si>
     <t>Onboarding — Skills Selection</t>
   </si>
   <si>
-    <t>React, Python, JavaScript, Node.js tags selected.</t>
-  </si>
-  <si>
     <t>Onboarding — Resume Upload &amp; Parse</t>
   </si>
   <si>
-    <t>Resume text submitted. Bypass AI clicked. Dashboard active.</t>
-  </si>
-  <si>
     <t>Dashboard Verification</t>
   </si>
   <si>
-    <t>Employability score element visible. Navigation bar confirmed.</t>
-  </si>
-  <si>
     <t>Scorecard Tab Navigation</t>
   </si>
   <si>
-    <t>Scorecard tab clicked. Score details and sub-tabs rendered.</t>
-  </si>
-  <si>
     <t>Simulation Sandbox Verification</t>
   </si>
   <si>
-    <t>Sandbox challenges rendered. Assessment cards visible.</t>
-  </si>
-  <si>
     <t>Profile &amp; Portfolio Manager</t>
   </si>
   <si>
-    <t>Profile tab opened. Credentials and Portfolio sections rendered.</t>
-  </si>
-  <si>
     <t>Settings Panel Verification</t>
   </si>
   <si>
-    <t>Settings tab opened. Configuration options displayed.</t>
-  </si>
-  <si>
     <t>Return to Home Dashboard</t>
-  </si>
-  <si>
-    <t>Home tab clicked. Dashboard with score summary re-rendered.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -190,7 +167,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF2E7D32"/>
+      <color rgb="FFC62828"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
@@ -202,8 +179,14 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF155724"/>
+      <color rgb="FF721C24"/>
       <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF721C24"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -213,7 +196,7 @@
       <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -227,12 +210,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD4EDDA"/>
+        <fgColor rgb="FFF8D7DA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F7FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -278,7 +266,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -290,9 +278,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -312,6 +297,24 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -688,20 +691,20 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="4">
         <v>13</v>
@@ -709,26 +712,26 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="5">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="B8" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="4">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="B9" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="6" t="s">
         <v>11</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -755,325 +758,325 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="10">
+        <v>25145</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="13">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="16">
+        <v>0</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="10">
+        <v>0</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="13">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="16">
+        <v>0</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="10">
+        <v>0</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="13">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="16">
+        <v>0</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="13">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="16">
+        <v>0</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="10">
+        <v>0</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="13">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="16">
+        <v>0</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="13">
         <v>12</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B13" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="16">
+        <v>0</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
         <v>13</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
-        <v>1</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="11">
-        <v>740</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
-        <v>2</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="11">
-        <v>1180</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
-        <v>3</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="11">
-        <v>95</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
-        <v>4</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="11">
-        <v>960</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
-        <v>5</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="11">
-        <v>880</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
-        <v>6</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="11">
-        <v>720</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="11">
-        <v>2200</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
-        <v>8</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="11">
-        <v>850</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
-        <v>9</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="11">
-        <v>1100</v>
-      </c>
-      <c r="F10" s="12" t="s">
+      <c r="B14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
-        <v>10</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="11">
-        <v>930</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
-        <v>11</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="11">
-        <v>870</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
-        <v>12</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="11">
-        <v>760</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
-        <v>13</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="11">
-        <v>680</v>
+      <c r="D14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="10">
+        <v>0</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>